<commit_message>
Harmonize Table S1/S2 group names with the manuscript and figures
Table S1 headers: MotX (trailing space), YvyF, Putative, FapA, Transglycosylase,
SwrB, FlgX, PilZ. parse_table_s1.py merges FliY into FliN under the name FliN
and drops the Flagellar_put alias, which the renamed header no longer needs.
ncbi_id_status_check.py gains --status-cache-input to reuse a saved NCBI
status snapshot. Rerun with the committed snapshot: all TP/FN/TPR values and
summary numbers unchanged, only names differ.
</commit_message>
<xml_diff>
--- a/code_and_data/pipeline_benchmarking/data/Table_S1.xlsx
+++ b/code_and_data/pipeline_benchmarking/data/Table_S1.xlsx
@@ -161,7 +161,7 @@
     <t>FlhF</t>
   </si>
   <si>
-    <t>PilZ/YcgR</t>
+    <t>PilZ</t>
   </si>
   <si>
     <t>FliT</t>
@@ -203,7 +203,7 @@
     <t>FlgR/FlrC/FlrA/FlaK/FlbD</t>
   </si>
   <si>
-    <t>SwrB/FlgW</t>
+    <t>SwrB</t>
   </si>
   <si>
     <t>SwrD</t>
@@ -212,10 +212,10 @@
     <t>FliY</t>
   </si>
   <si>
-    <t>Flagellar_put</t>
-  </si>
-  <si>
-    <t>yvyF</t>
+    <t>Putative</t>
+  </si>
+  <si>
+    <t>YvyF</t>
   </si>
   <si>
     <t>YviE/DUF6470</t>
@@ -233,7 +233,7 @@
     <t>MotK</t>
   </si>
   <si>
-    <t xml:space="preserve">MotX </t>
+    <t>MotX</t>
   </si>
   <si>
     <t>MotY</t>
@@ -269,7 +269,7 @@
     <t>FliZ</t>
   </si>
   <si>
-    <t>tPilZ/FlgX</t>
+    <t>FlgX</t>
   </si>
   <si>
     <t>FlhC</t>
@@ -281,7 +281,7 @@
     <t>DUF327</t>
   </si>
   <si>
-    <t>FapA/DUF342</t>
+    <t>FapA</t>
   </si>
   <si>
     <t>DUF1217</t>
@@ -314,7 +314,7 @@
     <t>FljA</t>
   </si>
   <si>
-    <t>SLT/Transglycosylase</t>
+    <t>Transglycosylase</t>
   </si>
   <si>
     <t>GCF_000092845.1</t>

</xml_diff>